<commit_message>
Sprint 6 en cero con el reparto por historia completa; Burndown S4-S5, ceremonias del S5 y plan de pruebas al dia
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/SIGMA_Burndown_Burnup.xlsx
+++ b/Fase 2/Evidencias Proyecto/SIGMA_Burndown_Burnup.xlsx
@@ -9158,7 +9158,7 @@
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
-          <t>1.1 · 22-09-2026 · Sprints 1 a 3 con registro diario</t>
+          <t>1.2 · 17-10-2026 · Sprints 1 a 5 con registro diario</t>
         </is>
       </c>
     </row>
@@ -10142,7 +10142,6 @@
       <c r="G18" s="19" t="n"/>
       <c r="H18" s="19" t="n"/>
     </row>
-    <row r="19"/>
     <row r="20" ht="15" customHeight="1" s="34">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -10205,7 +10204,6 @@
         <v/>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="34">
       <c r="A27" s="35" t="inlineStr">
         <is>
@@ -10214,8 +10212,6 @@
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="34"/>
-    <row r="29"/>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="44" t="inlineStr">
         <is>
@@ -10738,7 +10734,6 @@
       <c r="G17" s="19" t="n"/>
       <c r="H17" s="19" t="n"/>
     </row>
-    <row r="18"/>
     <row r="19" ht="15" customHeight="1" s="34">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -10801,7 +10796,6 @@
         <v/>
       </c>
     </row>
-    <row r="25"/>
     <row r="26" ht="15" customHeight="1" s="34">
       <c r="A26" s="35" t="inlineStr">
         <is>
@@ -11332,7 +11326,6 @@
       <c r="G17" s="19" t="n"/>
       <c r="H17" s="19" t="n"/>
     </row>
-    <row r="18"/>
     <row r="19" ht="15" customHeight="1" s="34">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -11395,7 +11388,6 @@
         <v/>
       </c>
     </row>
-    <row r="25"/>
     <row r="26" ht="15" customHeight="1" s="34">
       <c r="A26" s="35" t="inlineStr">
         <is>
@@ -11455,7 +11447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="34" min="1" max="1"/>
@@ -11597,7 +11589,9 @@
           <t>miércoles</t>
         </is>
       </c>
-      <c r="D8" s="28" t="n"/>
+      <c r="D8" s="28" t="n">
+        <v>23</v>
+      </c>
       <c r="E8" s="17">
         <f>$E7+$D8</f>
         <v/>
@@ -11631,7 +11625,9 @@
           <t>jueves</t>
         </is>
       </c>
-      <c r="D9" s="28" t="n"/>
+      <c r="D9" s="28" t="n">
+        <v>5</v>
+      </c>
       <c r="E9" s="13">
         <f>$E8+$D9</f>
         <v/>
@@ -11665,7 +11661,9 @@
           <t>viernes</t>
         </is>
       </c>
-      <c r="D10" s="28" t="n"/>
+      <c r="D10" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="E10" s="17">
         <f>$E9+$D10</f>
         <v/>
@@ -11699,7 +11697,9 @@
           <t>lunes</t>
         </is>
       </c>
-      <c r="D11" s="28" t="n"/>
+      <c r="D11" s="28" t="n">
+        <v>13</v>
+      </c>
       <c r="E11" s="13">
         <f>$E10+$D11</f>
         <v/>
@@ -11733,7 +11733,9 @@
           <t>martes</t>
         </is>
       </c>
-      <c r="D12" s="28" t="n"/>
+      <c r="D12" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="E12" s="17">
         <f>$E11+$D12</f>
         <v/>
@@ -11767,7 +11769,9 @@
           <t>miércoles</t>
         </is>
       </c>
-      <c r="D13" s="28" t="n"/>
+      <c r="D13" s="28" t="n">
+        <v>16</v>
+      </c>
       <c r="E13" s="13">
         <f>$E12+$D13</f>
         <v/>
@@ -11801,7 +11805,9 @@
           <t>jueves</t>
         </is>
       </c>
-      <c r="D14" s="28" t="n"/>
+      <c r="D14" s="28" t="n">
+        <v>5</v>
+      </c>
       <c r="E14" s="17">
         <f>$E13+$D14</f>
         <v/>
@@ -11835,7 +11841,9 @@
           <t>viernes</t>
         </is>
       </c>
-      <c r="D15" s="28" t="n"/>
+      <c r="D15" s="28" t="n">
+        <v>15</v>
+      </c>
       <c r="E15" s="13">
         <f>$E14+$D15</f>
         <v/>
@@ -11869,7 +11877,9 @@
           <t>lunes</t>
         </is>
       </c>
-      <c r="D16" s="28" t="n"/>
+      <c r="D16" s="28" t="n">
+        <v>32</v>
+      </c>
       <c r="E16" s="17">
         <f>$E15+$D16</f>
         <v/>
@@ -11903,7 +11913,9 @@
           <t>martes</t>
         </is>
       </c>
-      <c r="D17" s="28" t="n"/>
+      <c r="D17" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="E17" s="13">
         <f>$E16+$D17</f>
         <v/>
@@ -11942,6 +11954,7 @@
       <c r="G18" s="19" t="n"/>
       <c r="H18" s="19" t="n"/>
     </row>
+    <row r="19"/>
     <row r="20" ht="15" customHeight="1" s="34">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -12004,6 +12017,7 @@
         <v/>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="34">
       <c r="A27" s="35" t="inlineStr">
         <is>
@@ -12012,8 +12026,25 @@
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="34"/>
+    <row r="29">
+      <c r="A29" s="44" t="inlineStr">
+        <is>
+          <t>Estado al 17-10-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="34">
+      <c r="A30" s="45" t="inlineStr">
+        <is>
+          <t>Sprint cerrado en su alcance web: 19 historias y 109 puntos Terminada de los 148 comprometidos (SIGMA_Informe_Pruebas_Sprint_4.docx, 78 casos). Las cinco historias de aplicación móvil —HU-095, 103, 140, 141 y 160— se movieron al Sprint 6, por eso no queman aquí. Las historias nacieron con el trabajo repartido por módulo (planes, pauta y tareas) y se cerraron con sus pruebas el 01-10-2026. La columna amarilla se reconstruyó desde la Bitácora de Daily Scrum: cada historia quema sus puntos el último día en que el registro diario la nombra como trabajada, sin contar el día de la Sprint Review (ese día el equipo repasa todas para aceptarlas). Los puntos son los del Sprint Backlog y solo cuentan las historias Terminada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="34"/>
+    <row r="32" ht="15" customHeight="1" s="34"/>
+    <row r="33" ht="15" customHeight="1" s="34"/>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A21:B21"/>
@@ -12022,6 +12053,7 @@
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="A30:H33"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="A27:H28"/>
   </mergeCells>
@@ -12045,7 +12077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="34" min="1" max="1"/>
@@ -12187,7 +12219,9 @@
           <t>miércoles</t>
         </is>
       </c>
-      <c r="D8" s="28" t="n"/>
+      <c r="D8" s="28" t="n">
+        <v>5</v>
+      </c>
       <c r="E8" s="17">
         <f>$E7+$D8</f>
         <v/>
@@ -12221,7 +12255,9 @@
           <t>jueves</t>
         </is>
       </c>
-      <c r="D9" s="28" t="n"/>
+      <c r="D9" s="28" t="n">
+        <v>5</v>
+      </c>
       <c r="E9" s="13">
         <f>$E8+$D9</f>
         <v/>
@@ -12255,7 +12291,9 @@
           <t>viernes</t>
         </is>
       </c>
-      <c r="D10" s="28" t="n"/>
+      <c r="D10" s="28" t="n">
+        <v>0</v>
+      </c>
       <c r="E10" s="17">
         <f>$E9+$D10</f>
         <v/>
@@ -12289,7 +12327,9 @@
           <t>lunes</t>
         </is>
       </c>
-      <c r="D11" s="28" t="n"/>
+      <c r="D11" s="28" t="n">
+        <v>8</v>
+      </c>
       <c r="E11" s="13">
         <f>$E10+$D11</f>
         <v/>
@@ -12323,7 +12363,9 @@
           <t>martes</t>
         </is>
       </c>
-      <c r="D12" s="28" t="n"/>
+      <c r="D12" s="28" t="n">
+        <v>5</v>
+      </c>
       <c r="E12" s="17">
         <f>$E11+$D12</f>
         <v/>
@@ -12357,7 +12399,9 @@
           <t>miércoles</t>
         </is>
       </c>
-      <c r="D13" s="28" t="n"/>
+      <c r="D13" s="28" t="n">
+        <v>5</v>
+      </c>
       <c r="E13" s="13">
         <f>$E12+$D13</f>
         <v/>
@@ -12391,7 +12435,9 @@
           <t>jueves</t>
         </is>
       </c>
-      <c r="D14" s="28" t="n"/>
+      <c r="D14" s="28" t="n">
+        <v>3</v>
+      </c>
       <c r="E14" s="17">
         <f>$E13+$D14</f>
         <v/>
@@ -12425,7 +12471,9 @@
           <t>viernes</t>
         </is>
       </c>
-      <c r="D15" s="28" t="n"/>
+      <c r="D15" s="28" t="n">
+        <v>11</v>
+      </c>
       <c r="E15" s="13">
         <f>$E14+$D15</f>
         <v/>
@@ -12459,7 +12507,9 @@
           <t>lunes</t>
         </is>
       </c>
-      <c r="D16" s="28" t="n"/>
+      <c r="D16" s="28" t="n">
+        <v>10</v>
+      </c>
       <c r="E16" s="17">
         <f>$E15+$D16</f>
         <v/>
@@ -12493,7 +12543,9 @@
           <t>martes</t>
         </is>
       </c>
-      <c r="D17" s="28" t="n"/>
+      <c r="D17" s="28" t="n">
+        <v>98</v>
+      </c>
       <c r="E17" s="13">
         <f>$E16+$D17</f>
         <v/>
@@ -12532,6 +12584,7 @@
       <c r="G18" s="19" t="n"/>
       <c r="H18" s="19" t="n"/>
     </row>
+    <row r="19"/>
     <row r="20" ht="15" customHeight="1" s="34">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -12594,6 +12647,7 @@
         <v/>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="34">
       <c r="A27" s="35" t="inlineStr">
         <is>
@@ -12602,8 +12656,25 @@
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="34"/>
+    <row r="29">
+      <c r="A29" s="44" t="inlineStr">
+        <is>
+          <t>Estado al 17-10-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="34">
+      <c r="A30" s="45" t="inlineStr">
+        <is>
+          <t>Sprint cerrado en su alcance web: 26 historias y 150 puntos Terminada, 93 criterios verificados (SIGMA_Informe_Pruebas_Sprint_5.docx). Incluye las 12 historias que se incorporaron al Product Backlog durante el sprint (EP-21, SIGMA Twin y el inicio). Las 12 historias de la parte móvil —órdenes en terreno, sincronización, bitácora y voz— se movieron al Sprint 6. La columna amarilla se reconstruyó desde la Bitácora de Daily Scrum: cada historia quema sus puntos el último día en que el registro diario la nombra como trabajada, sin contar el día de la Sprint Review (ese día el equipo repasa todas para aceptarlas). Los puntos son los del Sprint Backlog y solo cuentan las historias Terminada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="34"/>
+    <row r="32" ht="15" customHeight="1" s="34"/>
+    <row r="33" ht="15" customHeight="1" s="34"/>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A21:B21"/>
@@ -12612,6 +12683,7 @@
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="A30:H33"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="A27:H28"/>
   </mergeCells>

</xml_diff>